<commit_message>
auto: 05-09 00:12 | .claude/settings.local.json "export_example_\345\205\250\351\207\217.xlsx" "export_example_\346\214\211\346\234\210_2026-05.xlsx" package-lock.json package.json scripts/gen_sample_xlsx.js src/utils/export.ts
</commit_message>
<xml_diff>
--- a/export_example_按月_2026-05.xlsx
+++ b/export_example_按月_2026-05.xlsx
@@ -1,30 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xiaoQAQhei\Desktop\家教课程账单_demo\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B490C48-66B6-455B-AA3C-F222FD83A771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="2026年5月 课程账单" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="2026年5月 课程账单" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="41">
   <si>
     <t>2026年5月 课程账单</t>
   </si>
   <si>
+    <t>李小明  ·  数学 150元/h · 物理 130元/h</t>
+  </si>
+  <si>
     <t>日期</t>
   </si>
   <si>
@@ -97,6 +91,9 @@
     <t>小计: 4节  8.0h  1160元</t>
   </si>
   <si>
+    <t>王雨涵  ·  英语 120元/h</t>
+  </si>
+  <si>
     <t>2026-05-04</t>
   </si>
   <si>
@@ -118,6 +115,9 @@
     <t>小计: 2节  4.0h  480元</t>
   </si>
   <si>
+    <t>陈子豪  ·  数学 160元/h</t>
+  </si>
+  <si>
     <t>2026-05-07</t>
   </si>
   <si>
@@ -134,48 +134,23 @@
   </si>
   <si>
     <t>总计: 8节课 | 16.0h | 2280元 | 已收 1160元 | 待收 1120元</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>李小明  ·  数学 150元/h · 物理 130元/h</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>王雨涵  ·  英语 120元/h</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>陈子豪  ·  数学 160元/h</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="宋体"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <color theme="9" tint="-0.249977111117893"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -187,8 +162,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFD1FAE5"/>
       </patternFill>
     </fill>
   </fills>
@@ -206,15 +180,17 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -547,313 +523,377 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G23"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12.4140625" customWidth="1"/>
-    <col min="3" max="3" width="13.9140625" customWidth="1"/>
-    <col min="6" max="6" width="10.33203125" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" t="s">
+        <v>5</v>
+      </c>
+      <c r="E12" t="s">
+        <v>6</v>
+      </c>
+      <c r="F12" t="s">
+        <v>7</v>
+      </c>
+      <c r="G12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>30</v>
+      </c>
+      <c r="F14" t="s">
+        <v>31</v>
+      </c>
+      <c r="G14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" t="s">
+        <v>4</v>
+      </c>
+      <c r="D18" t="s">
+        <v>5</v>
+      </c>
+      <c r="E18" t="s">
+        <v>6</v>
+      </c>
+      <c r="F18" t="s">
+        <v>7</v>
+      </c>
+      <c r="G18" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B20" t="s">
         <v>10</v>
       </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="C20" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" t="s">
-        <v>23</v>
-      </c>
-      <c r="G8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+      <c r="E20" t="s">
+        <v>37</v>
+      </c>
+      <c r="F20" t="s">
+        <v>31</v>
+      </c>
+      <c r="G20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B12" t="s">
-        <v>2</v>
-      </c>
-      <c r="C12" t="s">
-        <v>3</v>
-      </c>
-      <c r="D12" t="s">
-        <v>4</v>
-      </c>
-      <c r="E12" t="s">
-        <v>5</v>
-      </c>
-      <c r="F12" t="s">
-        <v>6</v>
-      </c>
-      <c r="G12" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" t="s">
-        <v>28</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" t="s">
-        <v>28</v>
-      </c>
-      <c r="F14" t="s">
-        <v>29</v>
-      </c>
-      <c r="G14" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+      <c r="B21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>1</v>
-      </c>
-      <c r="B18" t="s">
-        <v>2</v>
-      </c>
-      <c r="C18" t="s">
-        <v>3</v>
-      </c>
-      <c r="D18" t="s">
-        <v>4</v>
-      </c>
-      <c r="E18" t="s">
-        <v>5</v>
-      </c>
-      <c r="F18" t="s">
-        <v>6</v>
-      </c>
-      <c r="G18" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>32</v>
-      </c>
-      <c r="B19" t="s">
-        <v>9</v>
-      </c>
-      <c r="C19" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" t="s">
-        <v>34</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>35</v>
-      </c>
-      <c r="B20" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" t="s">
-        <v>33</v>
-      </c>
-      <c r="D20" t="s">
-        <v>11</v>
-      </c>
-      <c r="E20" t="s">
-        <v>34</v>
-      </c>
-      <c r="F20" t="s">
-        <v>29</v>
-      </c>
-      <c r="G20" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>37</v>
+      <c r="B23" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:G2 B23:F23 A10:G10 A9 A16:G16 A15 A22:G22 A21 A4:G8 B3:G3 A12:G14 B11:G11 A18:G20 B17:G17" numberStoredAsText="1"/>
-  </ignoredErrors>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
auto: 05-09 00:44 | "export_example_\346\214\211\346\234\210_2026-05.xlsx" scripts/gen_sample_xlsx.js
</commit_message>
<xml_diff>
--- a/export_example_按月_2026-05.xlsx
+++ b/export_example_按月_2026-05.xlsx
@@ -423,6 +423,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G23"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">

</xml_diff>

<commit_message>
auto: 05-09 01:35 | "export_example_\346\214\211\346\234\210_2026-05.xlsx" scripts/gen_sample_xlsx.js src/utils/export.ts
</commit_message>
<xml_diff>
--- a/export_example_按月_2026-05.xlsx
+++ b/export_example_按月_2026-05.xlsx
@@ -504,48 +504,48 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="str">
+      <c r="A5" s="4" t="str">
         <v>2026-05-03</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="4" t="str">
         <v>数学</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C5" s="4" t="str">
         <v>09:00-11:00</v>
       </c>
-      <c r="D5" s="2" t="str">
+      <c r="D5" s="4" t="str">
         <v>2h</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E5" s="4" t="str">
         <v>300元</v>
       </c>
-      <c r="F5" s="2" t="str">
+      <c r="F5" s="4" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G5" s="2" t="str">
+      <c r="G5" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="str">
+      <c r="A6" s="4" t="str">
         <v>2026-05-05</v>
       </c>
-      <c r="B6" s="2" t="str">
+      <c r="B6" s="4" t="str">
         <v>数学</v>
       </c>
-      <c r="C6" s="2" t="str">
+      <c r="C6" s="4" t="str">
         <v>09:00-11:00</v>
       </c>
-      <c r="D6" s="2" t="str">
+      <c r="D6" s="4" t="str">
         <v>2h</v>
       </c>
-      <c r="E6" s="2" t="str">
+      <c r="E6" s="4" t="str">
         <v>300元</v>
       </c>
-      <c r="F6" s="2" t="str">
+      <c r="F6" s="4" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G6" s="2" t="str">
+      <c r="G6" s="4" t="str">
         <v/>
       </c>
     </row>
@@ -647,25 +647,25 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="str">
+      <c r="A13" s="4" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="B13" s="2" t="str">
+      <c r="B13" s="4" t="str">
         <v>英语</v>
       </c>
-      <c r="C13" s="2" t="str">
+      <c r="C13" s="4" t="str">
         <v>16:00-18:00</v>
       </c>
-      <c r="D13" s="2" t="str">
+      <c r="D13" s="4" t="str">
         <v>2h</v>
       </c>
-      <c r="E13" s="2" t="str">
+      <c r="E13" s="4" t="str">
         <v>240元</v>
       </c>
-      <c r="F13" s="2" t="str">
+      <c r="F13" s="4" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G13" s="2" t="str">
+      <c r="G13" s="4" t="str">
         <v/>
       </c>
     </row>
@@ -744,25 +744,25 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="str">
+      <c r="A19" s="4" t="str">
         <v>2026-05-07</v>
       </c>
-      <c r="B19" s="2" t="str">
+      <c r="B19" s="4" t="str">
         <v>数学</v>
       </c>
-      <c r="C19" s="2" t="str">
+      <c r="C19" s="4" t="str">
         <v>10:00-12:00</v>
       </c>
-      <c r="D19" s="2" t="str">
+      <c r="D19" s="4" t="str">
         <v>2h</v>
       </c>
-      <c r="E19" s="2" t="str">
+      <c r="E19" s="4" t="str">
         <v>320元</v>
       </c>
-      <c r="F19" s="2" t="str">
+      <c r="F19" s="4" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G19" s="2" t="str">
+      <c r="G19" s="4" t="str">
         <v/>
       </c>
     </row>

</xml_diff>